<commit_message>
SAT-2-data-cleaning-and-preprocessing: Update processed data and anonymization notebook Step 1 completed
</commit_message>
<xml_diff>
--- a/Data/Processed Data/anonymized_SMSes_2025.xlsx
+++ b/Data/Processed Data/anonymized_SMSes_2025.xlsx
@@ -1900,7 +1900,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>23/12/2024</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>23/12/2024</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>23/12/2024</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>23/12/2024</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>23/12/2024</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>23/12/2024</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>24/12/2024</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>24/12/2024</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>24/12/2024</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>24/12/2024</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>25/12/2024</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>27/12/2024</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>27/12/2024</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>27/12/2024</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>28/12/2024</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>28/12/2024</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>28/12/2024</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -3119,7 +3119,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -3257,7 +3257,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3349,7 +3349,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3372,7 +3372,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -3510,7 +3510,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -3648,7 +3648,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -3809,7 +3809,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -3878,7 +3878,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -3970,7 +3970,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -4085,7 +4085,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -4177,7 +4177,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -4292,7 +4292,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>29/12/2024</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4315,7 +4315,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>30/12/2024</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>30/12/2024</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>30/12/2024</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -4384,7 +4384,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>30/12/2024</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>30/12/2024</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>30/12/2024</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -4453,7 +4453,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>30/12/2024</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>30/12/2024</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>30/12/2024</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>31/12/2024</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -4545,7 +4545,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>31/12/2024</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -4568,7 +4568,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>31/12/2024</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4591,7 +4591,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>31/12/2024</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>31/12/2024</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4637,7 +4637,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>31/12/2024</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>31/12/2024</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>&lt;DATE&gt;</t>
+          <t>31/12/2024</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">

</xml_diff>